<commit_message>
Open file previews nearly full-window, and show percentages as percentages
The preview dialog gets a 'full' size, 96% of the window up to 120rem, and
every preview fills its height: PDFs, Word, images, video, text, sheets
(tabs pinned to the bottom) and slide outlines. Markdown keeps a readable
line length inside it.

Spreadsheet cells with a percentage format showed the stored fraction
(0.654257142857143); they now show it as the format does (65.43%), for the
built-in 0% and 0.00% formats and custom ones, ignoring a % that only
appears in quoted text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/src/tests/fixtures/budget.xlsx
+++ b/frontend/src/tests/fixtures/budget.xlsx
@@ -51,9 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -422,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,9 +456,15 @@
       <c r="G1" s="1" t="n">
         <v>0.2583333333333334</v>
       </c>
+      <c r="H1" s="2" t="n">
+        <v>0.654257142857143</v>
+      </c>
+      <c r="I1" s="3" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Boat hire</t>
         </is>
@@ -467,7 +475,7 @@
       <c r="C2" t="n">
         <v>1200</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="5" t="n">
         <v>46321</v>
       </c>
       <c r="E2" t="b">
@@ -483,7 +491,7 @@
       <c r="C3" t="n">
         <v>340.3</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="6" t="n">
         <v>46323.60416666666</v>
       </c>
       <c r="E3" t="b">

</xml_diff>